<commit_message>
Small changes to Torre_Orsina params
</commit_message>
<xml_diff>
--- a/Torre_Orsina/Parameters/Site_Config_TC.xlsx
+++ b/Torre_Orsina/Parameters/Site_Config_TC.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="B:\group\pelligrp\Project_folders\MountainWater\Tethys_Chloris\Workflow_dev\Scripts\Cat\TeC_Source_Code\Torre_Orsina\Parameters\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F42EB8F6-10D2-4FF6-93BC-B8FF1D2AD557}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{99C32758-17C1-48A8-BE27-8B8449614085}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-5475" windowWidth="29040" windowHeight="17520" xr2:uid="{88CAB792-6FF5-4371-9CFE-4BFDB664029A}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{88CAB792-6FF5-4371-9CFE-4BFDB664029A}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>

</xml_diff>